<commit_message>
Add new metadata files and results for risk analysis runs
- Created `pareto_results_SA_sgAdaptive_b30_K20_risk_topsis_baseline.xlsx` to store baseline results.
- Added metadata for run `Run_20260608_114256_05ip_K20_Ekleme_risk_b30` with parameters and file references.
- Added metadata for run `Run_20260608_121454_13eps_K20_Ekleme_risk_b30` with parameters and logging information.
</commit_message>
<xml_diff>
--- a/results/models/coverage_v10_SA_ELECTRE_Baseline_SA_sgAdaptive_b30_K20_t0.15_risk.xlsx
+++ b/results/models/coverage_v10_SA_ELECTRE_Baseline_SA_sgAdaptive_b30_K20_t0.15_risk.xlsx
@@ -445,13 +445,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.4732437462688413</v>
+        <v>0.1522649086813897</v>
       </c>
       <c r="C2" t="n">
-        <v>1.101053719311412</v>
+        <v>2.167249975932604</v>
       </c>
       <c r="D2" t="n">
-        <v>1.574297465580253</v>
+        <v>2.319514884613994</v>
       </c>
     </row>
     <row r="3">
@@ -461,13 +461,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2.378752633374494</v>
+        <v>1.576911083281682</v>
       </c>
       <c r="C3" t="n">
-        <v>1.538600267351712</v>
+        <v>1.812326210363167</v>
       </c>
       <c r="D3" t="n">
-        <v>3.917352900726205</v>
+        <v>3.389237293644849</v>
       </c>
     </row>
     <row r="4">
@@ -477,13 +477,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2.626879587530645</v>
+        <v>1.832939778144957</v>
       </c>
       <c r="C4" t="n">
-        <v>1.741707851358834</v>
+        <v>1.863994119962391</v>
       </c>
       <c r="D4" t="n">
-        <v>4.368587438889479</v>
+        <v>3.696933898107348</v>
       </c>
     </row>
     <row r="5">
@@ -496,10 +496,10 @@
         <v>2.410374253683325</v>
       </c>
       <c r="C5" t="n">
-        <v>1.713914829665694</v>
+        <v>2.277862365166214</v>
       </c>
       <c r="D5" t="n">
-        <v>4.124289083349019</v>
+        <v>4.688236618849539</v>
       </c>
     </row>
     <row r="6">
@@ -509,13 +509,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2.558014036638986</v>
+        <v>1.642498751995788</v>
       </c>
       <c r="C6" t="n">
-        <v>0.7390124767098514</v>
+        <v>0.7390124767098512</v>
       </c>
       <c r="D6" t="n">
-        <v>3.297026513348837</v>
+        <v>2.381511228705639</v>
       </c>
     </row>
     <row r="7">
@@ -525,13 +525,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3.991934106426882</v>
+        <v>3.083853389286975</v>
       </c>
       <c r="C7" t="n">
-        <v>3.076087178354149</v>
+        <v>4.059011507255033</v>
       </c>
       <c r="D7" t="n">
-        <v>7.068021284781032</v>
+        <v>7.142864896542008</v>
       </c>
     </row>
     <row r="8">
@@ -541,13 +541,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2.925714726357789</v>
+        <v>2.753467862123725</v>
       </c>
       <c r="C8" t="n">
-        <v>2.336441652906073</v>
+        <v>2.986081793941858</v>
       </c>
       <c r="D8" t="n">
-        <v>5.262156379263862</v>
+        <v>5.739549656065583</v>
       </c>
     </row>
     <row r="9">
@@ -557,13 +557,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>3.001673083586974</v>
+        <v>1.773070411886394</v>
       </c>
       <c r="C9" t="n">
-        <v>1.854681469607223</v>
+        <v>2.93869868410314</v>
       </c>
       <c r="D9" t="n">
-        <v>4.856354553194198</v>
+        <v>4.711769095989535</v>
       </c>
     </row>
     <row r="10">
@@ -576,10 +576,10 @@
         <v>1.017033915823054</v>
       </c>
       <c r="C10" t="n">
-        <v>1.462805443545123</v>
+        <v>1.855662819958339</v>
       </c>
       <c r="D10" t="n">
-        <v>2.479839359368177</v>
+        <v>2.872696735781393</v>
       </c>
     </row>
     <row r="11">
@@ -589,13 +589,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>2.710231178354549</v>
+        <v>1.436589820550373</v>
       </c>
       <c r="C11" t="n">
-        <v>2.125467412362802</v>
+        <v>3.171272580117311</v>
       </c>
       <c r="D11" t="n">
-        <v>4.835698590717351</v>
+        <v>4.607862400667684</v>
       </c>
     </row>
     <row r="12">
@@ -621,13 +621,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2.58792557304611</v>
+        <v>2.261279516676049</v>
       </c>
       <c r="C13" t="n">
-        <v>0.8312385994267437</v>
+        <v>1.213620381246751</v>
       </c>
       <c r="D13" t="n">
-        <v>3.419164172472854</v>
+        <v>3.474899897922799</v>
       </c>
     </row>
     <row r="14">
@@ -640,10 +640,10 @@
         <v>2.960250971072124</v>
       </c>
       <c r="C14" t="n">
-        <v>1.707363134335014</v>
+        <v>2.301978819223848</v>
       </c>
       <c r="D14" t="n">
-        <v>4.667614105407138</v>
+        <v>5.262229790295972</v>
       </c>
     </row>
     <row r="15">
@@ -653,13 +653,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>3.451436896371884</v>
+        <v>2.480985033836274</v>
       </c>
       <c r="C15" t="n">
-        <v>2.749986061087136</v>
+        <v>3.329927286100637</v>
       </c>
       <c r="D15" t="n">
-        <v>6.20142295745902</v>
+        <v>5.810912319936912</v>
       </c>
     </row>
     <row r="16">
@@ -669,13 +669,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3.235407188995658</v>
+        <v>2.505845258649613</v>
       </c>
       <c r="C16" t="n">
-        <v>2.022335547565579</v>
+        <v>2.737708884854531</v>
       </c>
       <c r="D16" t="n">
-        <v>5.257742736561236</v>
+        <v>5.243554143504143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: stage all solver results, figures, metadata, and updated source files
- Add solver run outputs (metadata JSONs, coverage/IP/summary xlsx)
- Add generated figures (maps, charts) from recent solver runs
- Update log file and temp results
- Update src/14_single_stage.py, src/16_mclp.py, src/app_runner.py
- Add MCLP model outputs and single-stage results
</commit_message>
<xml_diff>
--- a/results/models/coverage_v10_SA_ELECTRE_Baseline_SA_sgAdaptive_b30_K20_t0.15_risk.xlsx
+++ b/results/models/coverage_v10_SA_ELECTRE_Baseline_SA_sgAdaptive_b30_K20_t0.15_risk.xlsx
@@ -445,13 +445,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1522649086813897</v>
+        <v>0.4732437462688413</v>
       </c>
       <c r="C2" t="n">
-        <v>2.167249975932604</v>
+        <v>1.101053719311412</v>
       </c>
       <c r="D2" t="n">
-        <v>2.319514884613994</v>
+        <v>1.574297465580253</v>
       </c>
     </row>
     <row r="3">
@@ -461,13 +461,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1.576911083281682</v>
+        <v>2.378752633374494</v>
       </c>
       <c r="C3" t="n">
-        <v>1.812326210363167</v>
+        <v>1.538600267351712</v>
       </c>
       <c r="D3" t="n">
-        <v>3.389237293644849</v>
+        <v>3.917352900726205</v>
       </c>
     </row>
     <row r="4">
@@ -477,13 +477,13 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1.832939778144957</v>
+        <v>2.626879587530645</v>
       </c>
       <c r="C4" t="n">
-        <v>1.863994119962391</v>
+        <v>1.741707851358834</v>
       </c>
       <c r="D4" t="n">
-        <v>3.696933898107348</v>
+        <v>4.368587438889479</v>
       </c>
     </row>
     <row r="5">
@@ -496,10 +496,10 @@
         <v>2.410374253683325</v>
       </c>
       <c r="C5" t="n">
-        <v>2.277862365166214</v>
+        <v>1.713914829665694</v>
       </c>
       <c r="D5" t="n">
-        <v>4.688236618849539</v>
+        <v>4.124289083349019</v>
       </c>
     </row>
     <row r="6">
@@ -509,13 +509,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1.642498751995788</v>
+        <v>2.558014036638986</v>
       </c>
       <c r="C6" t="n">
-        <v>0.7390124767098512</v>
+        <v>0.7390124767098514</v>
       </c>
       <c r="D6" t="n">
-        <v>2.381511228705639</v>
+        <v>3.297026513348837</v>
       </c>
     </row>
     <row r="7">
@@ -525,13 +525,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3.083853389286975</v>
+        <v>3.991934106426882</v>
       </c>
       <c r="C7" t="n">
-        <v>4.059011507255033</v>
+        <v>3.076087178354149</v>
       </c>
       <c r="D7" t="n">
-        <v>7.142864896542008</v>
+        <v>7.068021284781032</v>
       </c>
     </row>
     <row r="8">
@@ -541,13 +541,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2.753467862123725</v>
+        <v>2.925714726357789</v>
       </c>
       <c r="C8" t="n">
-        <v>2.986081793941858</v>
+        <v>2.336441652906073</v>
       </c>
       <c r="D8" t="n">
-        <v>5.739549656065583</v>
+        <v>5.262156379263862</v>
       </c>
     </row>
     <row r="9">
@@ -557,13 +557,13 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1.773070411886394</v>
+        <v>3.001673083586974</v>
       </c>
       <c r="C9" t="n">
-        <v>2.93869868410314</v>
+        <v>1.854681469607223</v>
       </c>
       <c r="D9" t="n">
-        <v>4.711769095989535</v>
+        <v>4.856354553194198</v>
       </c>
     </row>
     <row r="10">
@@ -576,10 +576,10 @@
         <v>1.017033915823054</v>
       </c>
       <c r="C10" t="n">
-        <v>1.855662819958339</v>
+        <v>1.462805443545123</v>
       </c>
       <c r="D10" t="n">
-        <v>2.872696735781393</v>
+        <v>2.479839359368177</v>
       </c>
     </row>
     <row r="11">
@@ -589,13 +589,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1.436589820550373</v>
+        <v>2.710231178354549</v>
       </c>
       <c r="C11" t="n">
-        <v>3.171272580117311</v>
+        <v>2.125467412362802</v>
       </c>
       <c r="D11" t="n">
-        <v>4.607862400667684</v>
+        <v>4.835698590717351</v>
       </c>
     </row>
     <row r="12">
@@ -621,13 +621,13 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2.261279516676049</v>
+        <v>2.58792557304611</v>
       </c>
       <c r="C13" t="n">
-        <v>1.213620381246751</v>
+        <v>0.8312385994267437</v>
       </c>
       <c r="D13" t="n">
-        <v>3.474899897922799</v>
+        <v>3.419164172472854</v>
       </c>
     </row>
     <row r="14">
@@ -640,10 +640,10 @@
         <v>2.960250971072124</v>
       </c>
       <c r="C14" t="n">
-        <v>2.301978819223848</v>
+        <v>1.707363134335014</v>
       </c>
       <c r="D14" t="n">
-        <v>5.262229790295972</v>
+        <v>4.667614105407138</v>
       </c>
     </row>
     <row r="15">
@@ -653,13 +653,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2.480985033836274</v>
+        <v>3.451436896371884</v>
       </c>
       <c r="C15" t="n">
-        <v>3.329927286100637</v>
+        <v>2.749986061087136</v>
       </c>
       <c r="D15" t="n">
-        <v>5.810912319936912</v>
+        <v>6.20142295745902</v>
       </c>
     </row>
     <row r="16">
@@ -669,13 +669,13 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>2.505845258649613</v>
+        <v>3.235407188995658</v>
       </c>
       <c r="C16" t="n">
-        <v>2.737708884854531</v>
+        <v>2.022335547565579</v>
       </c>
       <c r="D16" t="n">
-        <v>5.243554143504143</v>
+        <v>5.257742736561236</v>
       </c>
     </row>
   </sheetData>

</xml_diff>